<commit_message>
Add My Updated Code
</commit_message>
<xml_diff>
--- a/Jupyter_Files/ML/Git_Steps.xlsx
+++ b/Jupyter_Files/ML/Git_Steps.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyLearning\Python_WS\LMS_ProITBridge\Jupyter_Files\ML\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5E87C8E-4B9C-4500-B8A7-781B3314CC6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE1694A-4A70-45CA-A94F-E6B4003EF7B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
   <si>
     <t>Step</t>
   </si>
@@ -167,6 +167,9 @@
   </si>
   <si>
     <t>git log --oneline -n 5</t>
+  </si>
+  <si>
+    <t>Updated</t>
   </si>
 </sst>
 </file>
@@ -502,7 +505,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
@@ -758,6 +761,11 @@
         <v>29</v>
       </c>
     </row>
+    <row r="39" spans="1:3">
+      <c r="B39" t="s">
+        <v>43</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C8">
     <sortCondition ref="A1:A8"/>

</xml_diff>